<commit_message>
feat: crypto OHLC daily - Open/High/Low/Close per coin per hari
</commit_message>
<xml_diff>
--- a/data/harga_cpo.xlsx
+++ b/data/harga_cpo.xlsx
@@ -993,13 +993,13 @@
         </is>
       </c>
       <c r="B35" t="n">
-        <v>4500</v>
+        <v>4519</v>
       </c>
       <c r="C35" t="n">
-        <v>16875</v>
+        <v>16946</v>
       </c>
       <c r="D35" t="n">
-        <v>0.05</v>
+        <v>0.88</v>
       </c>
       <c r="E35" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
feat: filter/sort tanggal di tab Crypto & Emas + OHLC display
</commit_message>
<xml_diff>
--- a/data/harga_cpo.xlsx
+++ b/data/harga_cpo.xlsx
@@ -993,13 +993,13 @@
         </is>
       </c>
       <c r="B35" t="n">
-        <v>4519</v>
+        <v>4564</v>
       </c>
       <c r="C35" t="n">
-        <v>16946</v>
+        <v>17115</v>
       </c>
       <c r="D35" t="n">
-        <v>0.88</v>
+        <v>-1.56</v>
       </c>
       <c r="E35" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
fix: crypto table - remove empty IDR/MCap columns, add ETH/SOL 24h cols
</commit_message>
<xml_diff>
--- a/data/harga_cpo.xlsx
+++ b/data/harga_cpo.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E64"/>
+  <dimension ref="A1:E65"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1616,6 +1616,27 @@
         </is>
       </c>
     </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="B65" t="n">
+        <v>4483</v>
+      </c>
+      <c r="C65" t="n">
+        <v>4.483</v>
+      </c>
+      <c r="D65" t="n">
+        <v>-0.51</v>
+      </c>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>https://tradingeconomics.com/commodity/palm-oil</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
fix: overview cards - sembako shows available items, crypto shows sentiment, emas shows Rp spread
</commit_message>
<xml_diff>
--- a/data/harga_cpo.xlsx
+++ b/data/harga_cpo.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E65"/>
+  <dimension ref="A1:E66"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1637,6 +1637,27 @@
         </is>
       </c>
     </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="B66" t="n">
+        <v>4483</v>
+      </c>
+      <c r="C66" t="n">
+        <v>4.483</v>
+      </c>
+      <c r="D66" t="n">
+        <v>0</v>
+      </c>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>https://tradingeconomics.com/commodity/palm-oil</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
fix: sembako table crash - element ID mismatch mini-tepung vs mini-minyak, wrap overview cards in try-catch
</commit_message>
<xml_diff>
--- a/data/harga_cpo.xlsx
+++ b/data/harga_cpo.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E66"/>
+  <dimension ref="A1:E67"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1658,6 +1658,27 @@
         </is>
       </c>
     </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="B67" t="n">
+        <v>4483</v>
+      </c>
+      <c r="C67" t="n">
+        <v>4.483</v>
+      </c>
+      <c r="D67" t="n">
+        <v>0</v>
+      </c>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>https://tradingeconomics.com/commodity/palm-oil</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
fix: dedup_all 254 rows + add_row_to_excel date-exists check to prevent future dupes
</commit_message>
<xml_diff>
--- a/data/harga_cpo.xlsx
+++ b/data/harga_cpo.xlsx
@@ -453,7 +453,7 @@
         <v>4060</v>
       </c>
       <c r="C2" t="n">
-        <v>15225</v>
+        <v>73080</v>
       </c>
       <c r="D2" t="n">
         <v>-1.54</v>
@@ -474,7 +474,7 @@
         <v>4421</v>
       </c>
       <c r="C3" t="n">
-        <v>16579</v>
+        <v>79578</v>
       </c>
       <c r="D3" t="n">
         <v>1.77</v>
@@ -495,7 +495,7 @@
         <v>4381</v>
       </c>
       <c r="C4" t="n">
-        <v>16429</v>
+        <v>78858</v>
       </c>
       <c r="D4" t="n">
         <v>0.8</v>
@@ -516,7 +516,7 @@
         <v>4330</v>
       </c>
       <c r="C5" t="n">
-        <v>16020603</v>
+        <v>77940</v>
       </c>
       <c r="D5" t="n">
         <v>-2.1</v>
@@ -532,7 +532,7 @@
         <v>4209</v>
       </c>
       <c r="C6" t="n">
-        <v>15571887</v>
+        <v>75762</v>
       </c>
       <c r="D6" t="n">
         <v>-1.81</v>
@@ -548,7 +548,7 @@
         <v>4228</v>
       </c>
       <c r="C7" t="n">
-        <v>15643782</v>
+        <v>76104</v>
       </c>
       <c r="D7" t="n">
         <v>-1.52</v>
@@ -564,7 +564,7 @@
         <v>4191</v>
       </c>
       <c r="C8" t="n">
-        <v>15508137</v>
+        <v>75438</v>
       </c>
       <c r="D8" t="n">
         <v>-1.34</v>
@@ -580,7 +580,7 @@
         <v>4359</v>
       </c>
       <c r="C9" t="n">
-        <v>16128800</v>
+        <v>78462</v>
       </c>
       <c r="D9" t="n">
         <v>0.19</v>
@@ -596,7 +596,7 @@
         <v>4381</v>
       </c>
       <c r="C10" t="n">
-        <v>16208783</v>
+        <v>78858</v>
       </c>
       <c r="D10" t="n">
         <v>1.63</v>
@@ -612,7 +612,7 @@
         <v>4197</v>
       </c>
       <c r="C11" t="n">
-        <v>15528248</v>
+        <v>75546</v>
       </c>
       <c r="D11" t="n">
         <v>1.43</v>
@@ -628,7 +628,7 @@
         <v>4032</v>
       </c>
       <c r="C12" t="n">
-        <v>14918548</v>
+        <v>72576</v>
       </c>
       <c r="D12" t="n">
         <v>-2.34</v>
@@ -644,7 +644,7 @@
         <v>4343</v>
       </c>
       <c r="C13" t="n">
-        <v>16070189</v>
+        <v>78174</v>
       </c>
       <c r="D13" t="n">
         <v>1.07</v>
@@ -660,7 +660,7 @@
         <v>4234</v>
       </c>
       <c r="C14" t="n">
-        <v>15664769</v>
+        <v>76212</v>
       </c>
       <c r="D14" t="n">
         <v>-2.24</v>
@@ -676,7 +676,7 @@
         <v>4010</v>
       </c>
       <c r="C15" t="n">
-        <v>14837072</v>
+        <v>72180</v>
       </c>
       <c r="D15" t="n">
         <v>-1.05</v>
@@ -692,7 +692,7 @@
         <v>4202</v>
       </c>
       <c r="C16" t="n">
-        <v>15548293</v>
+        <v>75636</v>
       </c>
       <c r="D16" t="n">
         <v>-1.97</v>
@@ -708,7 +708,7 @@
         <v>4125</v>
       </c>
       <c r="C17" t="n">
-        <v>15263661</v>
+        <v>74250</v>
       </c>
       <c r="D17" t="n">
         <v>1.67</v>
@@ -724,7 +724,7 @@
         <v>4377</v>
       </c>
       <c r="C18" t="n">
-        <v>16196572</v>
+        <v>78786</v>
       </c>
       <c r="D18" t="n">
         <v>-0.08</v>
@@ -740,7 +740,7 @@
         <v>4261</v>
       </c>
       <c r="C19" t="n">
-        <v>15766733</v>
+        <v>76698</v>
       </c>
       <c r="D19" t="n">
         <v>0.32</v>
@@ -756,7 +756,7 @@
         <v>4168</v>
       </c>
       <c r="C20" t="n">
-        <v>15421454</v>
+        <v>75024</v>
       </c>
       <c r="D20" t="n">
         <v>-0.11</v>
@@ -772,7 +772,7 @@
         <v>4034</v>
       </c>
       <c r="C21" t="n">
-        <v>14925509</v>
+        <v>72612</v>
       </c>
       <c r="D21" t="n">
         <v>-2.21</v>
@@ -788,7 +788,7 @@
         <v>4043</v>
       </c>
       <c r="C22" t="n">
-        <v>14960655</v>
+        <v>72774</v>
       </c>
       <c r="D22" t="n">
         <v>1.47</v>
@@ -804,7 +804,7 @@
         <v>4168</v>
       </c>
       <c r="C23" t="n">
-        <v>15421816</v>
+        <v>75024</v>
       </c>
       <c r="D23" t="n">
         <v>-0.41</v>
@@ -820,7 +820,7 @@
         <v>4105</v>
       </c>
       <c r="C24" t="n">
-        <v>15190349</v>
+        <v>73890</v>
       </c>
       <c r="D24" t="n">
         <v>-0.83</v>
@@ -836,7 +836,7 @@
         <v>4029</v>
       </c>
       <c r="C25" t="n">
-        <v>14908960</v>
+        <v>72522</v>
       </c>
       <c r="D25" t="n">
         <v>-0.84</v>
@@ -852,7 +852,7 @@
         <v>4093</v>
       </c>
       <c r="C26" t="n">
-        <v>15142314</v>
+        <v>73674</v>
       </c>
       <c r="D26" t="n">
         <v>-2.24</v>
@@ -868,7 +868,7 @@
         <v>4082</v>
       </c>
       <c r="C27" t="n">
-        <v>15101861</v>
+        <v>73476</v>
       </c>
       <c r="D27" t="n">
         <v>-1.55</v>
@@ -884,7 +884,7 @@
         <v>4360</v>
       </c>
       <c r="C28" t="n">
-        <v>16133261</v>
+        <v>78480</v>
       </c>
       <c r="D28" t="n">
         <v>-0.01</v>
@@ -900,7 +900,7 @@
         <v>4289</v>
       </c>
       <c r="C29" t="n">
-        <v>15869112</v>
+        <v>77202</v>
       </c>
       <c r="D29" t="n">
         <v>1.19</v>
@@ -916,7 +916,7 @@
         <v>4183</v>
       </c>
       <c r="C30" t="n">
-        <v>15478214</v>
+        <v>75294</v>
       </c>
       <c r="D30" t="n">
         <v>-2.39</v>
@@ -932,7 +932,7 @@
         <v>4219</v>
       </c>
       <c r="C31" t="n">
-        <v>15610292</v>
+        <v>75942</v>
       </c>
       <c r="D31" t="n">
         <v>0.22</v>
@@ -948,7 +948,7 @@
         <v>4293</v>
       </c>
       <c r="C32" t="n">
-        <v>15882660</v>
+        <v>77274</v>
       </c>
       <c r="D32" t="n">
         <v>-1.06</v>
@@ -964,7 +964,7 @@
         <v>4104</v>
       </c>
       <c r="C33" t="n">
-        <v>15183836</v>
+        <v>73872</v>
       </c>
       <c r="D33" t="n">
         <v>1.36</v>
@@ -980,7 +980,7 @@
         <v>4252</v>
       </c>
       <c r="C34" t="n">
-        <v>15733594</v>
+        <v>76536</v>
       </c>
       <c r="D34" t="n">
         <v>-2.21</v>
@@ -996,7 +996,7 @@
         <v>4515</v>
       </c>
       <c r="C35" t="n">
-        <v>16931</v>
+        <v>81270</v>
       </c>
       <c r="D35" t="n">
         <v>-0.42</v>
@@ -1017,7 +1017,7 @@
         <v>5068</v>
       </c>
       <c r="C36" t="n">
-        <v>19005</v>
+        <v>91224</v>
       </c>
       <c r="D36" t="n">
         <v>-1.91</v>
@@ -1038,7 +1038,7 @@
         <v>4480</v>
       </c>
       <c r="C37" t="n">
-        <v>4.48</v>
+        <v>80640</v>
       </c>
       <c r="D37" t="n">
         <v>0</v>
@@ -1059,7 +1059,7 @@
         <v>4480</v>
       </c>
       <c r="C38" t="n">
-        <v>4.48</v>
+        <v>80640</v>
       </c>
       <c r="D38" t="n">
         <v>0</v>

</xml_diff>